<commit_message>
Replace all August 2026 labels across all calculation sheets, RCM and ITC rows with target month
</commit_message>
<xml_diff>
--- a/output/GSTR-1_SEP-26_AUTOMATED.xlsx
+++ b/output/GSTR-1_SEP-26_AUTOMATED.xlsx
@@ -7901,9 +7901,12 @@
         <v/>
       </c>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="E54" s="985" t="n"/>
     </row>
+    <row r="55"/>
+    <row r="56"/>
     <row r="57">
       <c r="C57">
         <f>+CELL("filename")</f>
@@ -8827,7 +8830,7 @@
     <row r="16" ht="15.75" customHeight="1" thickBot="1">
       <c r="A16" s="1082" t="inlineStr">
         <is>
-          <t xml:space="preserve">                  GST PAYABLE UNDER RCM FOR THE MONTH OF AUG-26</t>
+          <t xml:space="preserve">                  GST PAYABLE UNDER RCM FOR THE MONTH OF SEP-26</t>
         </is>
       </c>
       <c r="B16" s="972" t="n"/>
@@ -8994,7 +8997,7 @@
     <row r="23">
       <c r="A23" s="1216" t="inlineStr">
         <is>
-          <t>Security Services (AUG-25 TO AUG-26)</t>
+          <t>Security Services (AUG-25 TO SEP-26)</t>
         </is>
       </c>
       <c r="B23" s="1183" t="n"/>
@@ -9124,7 +9127,7 @@
     <row r="28" ht="15.75" customHeight="1" thickBot="1">
       <c r="A28" s="1082" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    INELIGIBLE CREDIT FOR THE MONTH OF AUG-26</t>
+          <t xml:space="preserve">                    INELIGIBLE CREDIT FOR THE MONTH OF SEP-26</t>
         </is>
       </c>
       <c r="B28" s="972" t="n"/>
@@ -9204,7 +9207,7 @@
     <row r="32">
       <c r="A32" s="1061" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ITC FOR THE  AUG-26</t>
+          <t xml:space="preserve"> ITC FOR THE  SEP-26</t>
         </is>
       </c>
       <c r="B32" s="1069" t="n"/>
@@ -9408,7 +9411,7 @@
     <row r="41" ht="15.75" customHeight="1" thickBot="1">
       <c r="A41" s="1082" t="inlineStr">
         <is>
-          <t xml:space="preserve">                GST Payable for the month of AUG-26</t>
+          <t xml:space="preserve">                GST Payable for the month of SEP-26</t>
         </is>
       </c>
       <c r="B41" s="972" t="n"/>
@@ -13032,7 +13035,7 @@
     <row r="52" ht="15.75" customHeight="1" thickBot="1">
       <c r="A52" s="1369" t="inlineStr">
         <is>
-          <t xml:space="preserve">                  GST PAYABLE UNDER RCM FOR THE MONTH OF AUG-26</t>
+          <t xml:space="preserve">                  GST PAYABLE UNDER RCM FOR THE MONTH OF SEP-26</t>
         </is>
       </c>
       <c r="B52" s="972" t="n"/>
@@ -13319,7 +13322,7 @@
     <row r="68" ht="15.75" customHeight="1" thickBot="1">
       <c r="A68" s="1369" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    INPUT TAX CREDIT FOR THE MONTH OF AUG-26</t>
+          <t xml:space="preserve">                    INPUT TAX CREDIT FOR THE MONTH OF SEP-26</t>
         </is>
       </c>
       <c r="B68" s="972" t="n"/>
@@ -13403,7 +13406,7 @@
     <row r="73">
       <c r="A73" s="1061" t="inlineStr">
         <is>
-          <t>Add : ITC FOR THE AUG-26</t>
+          <t>Add : ITC FOR THE SEP-26</t>
         </is>
       </c>
       <c r="B73" s="1069">
@@ -13448,7 +13451,7 @@
     <row r="75">
       <c r="A75" s="1061" t="inlineStr">
         <is>
-          <t>Add : ITC of RCM of AUG-26</t>
+          <t>Add : ITC of RCM of SEP-26</t>
         </is>
       </c>
       <c r="B75" s="1069">
@@ -13651,7 +13654,7 @@
     <row r="85">
       <c r="A85" s="1061" t="inlineStr">
         <is>
-          <t>Less : ITC OF IGST Utilized for AUG-26</t>
+          <t>Less : ITC OF IGST Utilized for SEP-26</t>
         </is>
       </c>
       <c r="B85" s="1069">
@@ -13674,7 +13677,7 @@
     <row r="86">
       <c r="A86" s="1061" t="inlineStr">
         <is>
-          <t>Less : ITC Utilised FOR the AUG-26</t>
+          <t>Less : ITC Utilised FOR the SEP-26</t>
         </is>
       </c>
       <c r="B86" s="1069">
@@ -13772,7 +13775,7 @@
     <row r="91" ht="15.75" customHeight="1" thickBot="1">
       <c r="A91" s="1369" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    INELIGIBLE CREDIT FOR THE MONTH OF AUG-26</t>
+          <t xml:space="preserve">                    INELIGIBLE CREDIT FOR THE MONTH OF SEP-26</t>
         </is>
       </c>
       <c r="B91" s="972" t="n"/>
@@ -13865,7 +13868,7 @@
     <row r="95">
       <c r="A95" s="1061" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ITC FOR THE AUG-26 Including RCM ( Atmoshphere ,Footprint  &amp; SUN PARK WEST)</t>
+          <t xml:space="preserve"> ITC FOR THE SEP-26 Including RCM ( Atmoshphere ,Footprint  &amp; SUN PARK WEST)</t>
         </is>
       </c>
       <c r="B95" s="1069">
@@ -13975,7 +13978,7 @@
     <row r="100" ht="15.75" customHeight="1" thickBot="1">
       <c r="A100" s="1369" t="inlineStr">
         <is>
-          <t xml:space="preserve">                GST Payable for the month of AUG-26</t>
+          <t xml:space="preserve">                GST Payable for the month of SEP-26</t>
         </is>
       </c>
       <c r="B100" s="972" t="n"/>
@@ -14985,6 +14988,12 @@
       <c r="B168" s="330" t="n"/>
       <c r="F168" s="1394" t="n"/>
     </row>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
     <row r="175">
       <c r="A175" s="1">
         <f>+'SUN REALTY ATMOS-CALC'!A92</f>
@@ -15477,7 +15486,7 @@
         <v>5</v>
       </c>
       <c r="B36" s="268" t="n">
-        <v>46285</v>
+        <v>46295</v>
       </c>
       <c r="C36" s="269" t="inlineStr">
         <is>
@@ -15860,6 +15869,7 @@
       <c r="D65" s="1403" t="n"/>
       <c r="E65" s="1403" t="n"/>
     </row>
+    <row r="66"/>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
@@ -27660,7 +27670,7 @@
     <row r="41" ht="15" customHeight="1" thickBot="1">
       <c r="A41" s="1045" t="inlineStr">
         <is>
-          <t xml:space="preserve">                  GST PAYABLE UNDER RCM FOR THE MONTH OF AUG-26</t>
+          <t xml:space="preserve">                  GST PAYABLE UNDER RCM FOR THE MONTH OF SEP-26</t>
         </is>
       </c>
       <c r="B41" s="972" t="n"/>
@@ -27950,7 +27960,7 @@
     <row r="57" ht="15" customHeight="1" thickBot="1">
       <c r="A57" s="1045" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    INPUT TAX CREDIT FOR THE MONTH OF AUG-26</t>
+          <t xml:space="preserve">                    INPUT TAX CREDIT FOR THE MONTH OF SEP-26</t>
         </is>
       </c>
       <c r="B57" s="972" t="n"/>
@@ -28029,7 +28039,7 @@
     <row r="62">
       <c r="A62" s="1061" t="inlineStr">
         <is>
-          <t>Add : ITC FOR THE AUG-26</t>
+          <t>Add : ITC FOR THE SEP-26</t>
         </is>
       </c>
       <c r="B62" s="1065" t="n">
@@ -28306,7 +28316,7 @@
     <row r="77" ht="15" customHeight="1" thickBot="1">
       <c r="A77" s="1082" t="inlineStr">
         <is>
-          <t xml:space="preserve">                GST Payable for the month of AUG-26</t>
+          <t xml:space="preserve">                GST Payable for the month of SEP-26</t>
         </is>
       </c>
       <c r="B77" s="972" t="n"/>
@@ -28645,7 +28655,7 @@
     <row r="99">
       <c r="A99" s="548" t="inlineStr">
         <is>
-          <t>Total Input Tax Credit Available for the AUG-26</t>
+          <t>Total Input Tax Credit Available for the SEP-26</t>
         </is>
       </c>
       <c r="B99" s="1089">
@@ -28738,7 +28748,7 @@
     <row r="103" ht="15" customHeight="1" thickBot="1">
       <c r="A103" s="545" t="inlineStr">
         <is>
-          <t>Total Input Tax Credit for the AUG-26</t>
+          <t>Total Input Tax Credit for the SEP-26</t>
         </is>
       </c>
       <c r="B103" s="1093">
@@ -28761,6 +28771,20 @@
     <row r="104">
       <c r="B104" s="1007" t="n"/>
     </row>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
     <row r="119">
       <c r="A119" s="525">
         <f>+'SUN REALTY-MEM COLL'!C57</f>
@@ -29252,6 +29276,8 @@
       <c r="C36" s="235" t="n"/>
       <c r="D36" s="1403" t="n"/>
     </row>
+    <row r="37"/>
+    <row r="38"/>
     <row r="39">
       <c r="E39" s="1403" t="n"/>
     </row>
@@ -30582,6 +30608,7 @@
       </c>
       <c r="G12" s="86" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="961" t="inlineStr">
         <is>
@@ -30589,6 +30616,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="112" t="inlineStr">
         <is>
@@ -35903,6 +35931,7 @@
         <v/>
       </c>
     </row>
+    <row r="105"/>
     <row r="106" ht="17.25" customHeight="1">
       <c r="C106" s="1112" t="n"/>
       <c r="D106" s="1113">
@@ -35963,13 +35992,17 @@
       <c r="K112" s="310" t="n"/>
       <c r="L112" s="311" t="n"/>
     </row>
+    <row r="113"/>
     <row r="114">
       <c r="F114" s="1098" t="n"/>
     </row>
+    <row r="115"/>
     <row r="116">
       <c r="B116" s="312" t="n"/>
       <c r="C116" s="305" t="n"/>
     </row>
+    <row r="117"/>
+    <row r="118"/>
     <row r="119">
       <c r="B119" s="884" t="n"/>
     </row>
@@ -48950,7 +48983,7 @@
     <row r="43" ht="15" customHeight="1" thickBot="1">
       <c r="A43" s="1153" t="inlineStr">
         <is>
-          <t xml:space="preserve">                  GST PAYABLE UNDER RCM FOR THE MONTH OF  AUG-26</t>
+          <t xml:space="preserve">                  GST PAYABLE UNDER RCM FOR THE MONTH OF  SEP-26</t>
         </is>
       </c>
       <c r="B43" s="1154" t="n"/>
@@ -49169,7 +49202,7 @@
     <row r="55" ht="15" customHeight="1" thickBot="1">
       <c r="A55" s="1172" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    INELIGIBLE CREDIT FOR THE MONTH OF AUG-26</t>
+          <t xml:space="preserve">                    INELIGIBLE CREDIT FOR THE MONTH OF SEP-26</t>
         </is>
       </c>
       <c r="B55" s="969" t="n"/>
@@ -49229,7 +49262,7 @@
     <row r="59">
       <c r="A59" s="1176" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ITC FOR THE AUG-26</t>
+          <t xml:space="preserve"> ITC FOR THE SEP-26</t>
         </is>
       </c>
       <c r="B59" s="1177" t="n">
@@ -49337,10 +49370,11 @@
       <c r="G64" s="991" t="n"/>
       <c r="H64" s="991" t="n"/>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" s="1082" t="inlineStr">
         <is>
-          <t xml:space="preserve">                GST Payable for the month of AUG-26</t>
+          <t xml:space="preserve">                GST Payable for the month of SEP-26</t>
         </is>
       </c>
       <c r="B66" s="972" t="n"/>
@@ -49527,6 +49561,8 @@
       <c r="F78" s="440" t="n"/>
       <c r="G78" s="1007" t="n"/>
     </row>
+    <row r="79"/>
+    <row r="80"/>
     <row r="81">
       <c r="A81" s="398" t="n"/>
       <c r="B81" s="398" t="n"/>
@@ -49540,6 +49576,7 @@
       <c r="D82" s="331" t="n"/>
       <c r="E82" s="330" t="n"/>
     </row>
+    <row r="83"/>
     <row r="84">
       <c r="B84" s="330" t="n"/>
       <c r="C84" s="330" t="n"/>
@@ -49574,6 +49611,8 @@
       <c r="C89" s="442" t="n"/>
       <c r="D89" s="442" t="n"/>
     </row>
+    <row r="90"/>
+    <row r="91"/>
     <row r="92">
       <c r="A92" s="802">
         <f>+'SUN REALTY ATMOS-MEMBERS COLL'!B112</f>
@@ -56444,6 +56483,7 @@
         <v/>
       </c>
     </row>
+    <row r="231"/>
     <row r="232" ht="18.75" customHeight="1">
       <c r="B232" s="1201" t="inlineStr">
         <is>
@@ -56468,6 +56508,7 @@
         <v/>
       </c>
     </row>
+    <row r="234"/>
     <row r="235">
       <c r="A235">
         <f>+'SUN REALTY-CALC'!A119</f>
@@ -57319,7 +57360,7 @@
     <row r="44" ht="15" customHeight="1" thickBot="1">
       <c r="A44" s="1082" t="inlineStr">
         <is>
-          <t xml:space="preserve">                GST Payable for the month of AUG'26</t>
+          <t xml:space="preserve">                GST Payable for the month of SEP'26</t>
         </is>
       </c>
       <c r="B44" s="972" t="n"/>
@@ -57506,15 +57547,116 @@
       <c r="F56" s="440" t="n"/>
       <c r="G56" s="1007" t="n"/>
     </row>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="1">
         <f>+'SUN REALTY ATMOS-MEMBERS COLL'!B112</f>
         <v/>
       </c>
     </row>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
     <row r="103">
       <c r="H103" s="1007" t="n"/>
     </row>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
     <row r="160">
       <c r="O160" s="1">
         <f>9957</f>
@@ -59940,6 +60082,7 @@
         <v/>
       </c>
     </row>
+    <row r="98"/>
     <row r="99" ht="15.75" customHeight="1">
       <c r="B99" s="1243" t="inlineStr">
         <is>
@@ -59965,6 +60108,7 @@
         <v/>
       </c>
     </row>
+    <row r="101"/>
     <row r="102">
       <c r="A102">
         <f>+'SUN REALTY-CALC'!A119</f>
@@ -60469,7 +60613,7 @@
     <row r="19" ht="15" customHeight="1" thickBot="1">
       <c r="A19" s="1082" t="inlineStr">
         <is>
-          <t xml:space="preserve">                  GST PAYABLE UNDER RCM FOR THE MONTH OF AUG'26</t>
+          <t xml:space="preserve">                  GST PAYABLE UNDER RCM FOR THE MONTH OF SEP'26</t>
         </is>
       </c>
       <c r="B19" s="972" t="n"/>
@@ -60773,7 +60917,7 @@
     <row r="31" ht="15" customHeight="1" thickBot="1">
       <c r="A31" s="1082" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    INELIGIBLE CREDIT FOR THE MONTH OF AUG'26</t>
+          <t xml:space="preserve">                    INELIGIBLE CREDIT FOR THE MONTH OF SEP'26</t>
         </is>
       </c>
       <c r="B31" s="972" t="n"/>
@@ -60833,7 +60977,7 @@
     <row r="35">
       <c r="A35" s="1061" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ITC FOR THE  AUG-26</t>
+          <t xml:space="preserve"> ITC FOR THE  SEP-26</t>
         </is>
       </c>
       <c r="B35" s="1069" t="n"/>
@@ -60987,7 +61131,7 @@
     <row r="44" ht="15" customHeight="1" thickBot="1">
       <c r="A44" s="1082" t="inlineStr">
         <is>
-          <t xml:space="preserve">                GST Payable for the month of AUG'26</t>
+          <t xml:space="preserve">                GST Payable for the month of SEP'26</t>
         </is>
       </c>
       <c r="B44" s="972" t="n"/>
@@ -61174,6 +61318,7 @@
       <c r="F56" s="440" t="n"/>
       <c r="G56" s="1007" t="n"/>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" s="330" t="n"/>
       <c r="B58" s="330" t="n"/>
@@ -61218,6 +61363,7 @@
       <c r="D61" s="612" t="n"/>
       <c r="E61" s="612" t="n"/>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" s="330" t="n"/>
       <c r="B63" s="330" t="n"/>
@@ -61229,15 +61375,46 @@
       <c r="C64" s="330" t="n"/>
       <c r="D64" s="330" t="n"/>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="B66" s="330" t="n"/>
     </row>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
     <row r="78">
       <c r="H78" s="1">
         <f>127214-1238</f>
         <v/>
       </c>
     </row>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
     <row r="98">
       <c r="M98" s="1">
         <f>7957235-6059</f>

</xml_diff>